<commit_message>
optimización actualizacion condiciones comerciales
</commit_message>
<xml_diff>
--- a/viveprop-platform/data/condiciones_cc_unified.xlsx
+++ b/viveprop-platform/data/condiciones_cc_unified.xlsx
@@ -415,26 +415,6 @@
   </sheetPr>
   <dimension ref="A1:R79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="50" customWidth="1" min="18" max="18"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -654,9 +634,12 @@
       <c r="L3" t="n">
         <v>10</v>
       </c>
+      <c r="M3" t="n">
+        <v>8</v>
+      </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2.028</t>
+          <t>2028</t>
         </is>
       </c>
     </row>
@@ -686,7 +669,7 @@
         <v>100000</v>
       </c>
       <c r="J4" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K4" t="n">
         <v>2</v>
@@ -694,9 +677,12 @@
       <c r="L4" t="n">
         <v>10</v>
       </c>
+      <c r="M4" t="n">
+        <v>8</v>
+      </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2.029</t>
+          <t>2029</t>
         </is>
       </c>
     </row>
@@ -708,16 +694,16 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>MAESTRA</t>
+          <t>INGEVEC</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SERRANO TORRE A</t>
+          <t>Serrano (SER)</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G5" t="n">
         <v>10</v>
@@ -726,7 +712,7 @@
         <v>100000</v>
       </c>
       <c r="J5" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
         <v>2</v>
@@ -734,9 +720,20 @@
       <c r="L5" t="n">
         <v>10</v>
       </c>
+      <c r="M5" t="n">
+        <v>8</v>
+      </c>
+      <c r="N5" t="n">
+        <v>10</v>
+      </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2.028</t>
+          <t>Entrega Inmediata</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Crédito y arriendo garantizado en paralaleo hasta el 30/06/2031)</t>
         </is>
       </c>
     </row>
@@ -766,7 +763,7 @@
         <v>100000</v>
       </c>
       <c r="J6" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="K6" t="n">
         <v>1</v>
@@ -774,9 +771,12 @@
       <c r="L6" t="n">
         <v>10</v>
       </c>
+      <c r="M6" t="n">
+        <v>9</v>
+      </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2.029</t>
+          <t>2029</t>
         </is>
       </c>
     </row>
@@ -802,6 +802,11 @@
       <c r="E7" t="n">
         <v>2</v>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>SurOriente</t>
+        </is>
+      </c>
       <c r="G7" t="n">
         <v>10</v>
       </c>
@@ -809,7 +814,7 @@
         <v>100000</v>
       </c>
       <c r="J7" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="K7" t="n">
         <v>2</v>
@@ -817,9 +822,12 @@
       <c r="L7" t="n">
         <v>10</v>
       </c>
+      <c r="M7" t="n">
+        <v>8</v>
+      </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2.029</t>
+          <t>2029</t>
         </is>
       </c>
     </row>
@@ -849,7 +857,7 @@
         <v>100000</v>
       </c>
       <c r="J8" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="K8" t="n">
         <v>1</v>
@@ -857,9 +865,12 @@
       <c r="L8" t="n">
         <v>10</v>
       </c>
+      <c r="M8" t="n">
+        <v>9</v>
+      </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2.029</t>
+          <t>2029</t>
         </is>
       </c>
     </row>
@@ -876,11 +887,28 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Pintor Cicarelli I: solo tipología 3D1B (con descuento máximo de venta de 10%)</t>
-        </is>
+          <t>Pintor Cicarelli I (PC I)</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>13</v>
+      </c>
+      <c r="G9" t="n">
+        <v>15</v>
       </c>
       <c r="H9" t="n">
         <v>100000</v>
+      </c>
+      <c r="J9" t="n">
+        <v>4</v>
+      </c>
+      <c r="M9" t="n">
+        <v>5</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Pre-entrega</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -922,6 +950,9 @@
       <c r="L10" t="n">
         <v>10</v>
       </c>
+      <c r="M10" t="n">
+        <v>10</v>
+      </c>
       <c r="P10" t="inlineStr">
         <is>
           <t>Inmediata</t>
@@ -959,6 +990,9 @@
       <c r="L11" t="n">
         <v>10</v>
       </c>
+      <c r="M11" t="n">
+        <v>10</v>
+      </c>
       <c r="P11" t="inlineStr">
         <is>
           <t>Inmediata</t>
@@ -978,11 +1012,28 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Jardines de Alvarado: solo tipología 3D1B (con descuento máximo de venta de 10%)</t>
-        </is>
+          <t>Jardines de Alvarado</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>15</v>
+      </c>
+      <c r="G12" t="n">
+        <v>10</v>
       </c>
       <c r="H12" t="n">
         <v>100000</v>
+      </c>
+      <c r="J12" t="n">
+        <v>60</v>
+      </c>
+      <c r="M12" t="n">
+        <v>10</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Inmediata</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -998,11 +1049,36 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Mirador Mapocho: solo tipología 1D1B (con descuento máximo de venta de 10%)</t>
-        </is>
+          <t>Mirador Mapocho</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>10</v>
+      </c>
+      <c r="E13" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>1D</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>10</v>
       </c>
       <c r="H13" t="n">
         <v>100000</v>
+      </c>
+      <c r="J13" t="n">
+        <v>60</v>
+      </c>
+      <c r="M13" t="n">
+        <v>10</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Inmediata</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -1022,7 +1098,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G14" t="n">
         <v>10</v>
@@ -1036,6 +1112,9 @@
       <c r="L14" t="n">
         <v>10</v>
       </c>
+      <c r="M14" t="n">
+        <v>10</v>
+      </c>
       <c r="P14" t="inlineStr">
         <is>
           <t>Inmediata</t>
@@ -1073,6 +1152,9 @@
       <c r="L15" t="n">
         <v>10</v>
       </c>
+      <c r="M15" t="n">
+        <v>10</v>
+      </c>
       <c r="P15" t="inlineStr">
         <is>
           <t>Inmediata</t>
@@ -1110,6 +1192,9 @@
       <c r="L16" t="n">
         <v>10</v>
       </c>
+      <c r="M16" t="n">
+        <v>10</v>
+      </c>
       <c r="P16" t="inlineStr">
         <is>
           <t>Inmediata</t>
@@ -1129,11 +1214,33 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Plaza Quilicura: Se deben vender todos los departamentos con estacionamiento de manera obligatoria; Estacionamientos bajan a UF 250 (Precio anterior UF 290)</t>
-        </is>
+          <t>Plaza Quilicura</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>12</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Solo 2D (36m2)</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>10</v>
       </c>
       <c r="H17" t="n">
         <v>100000</v>
+      </c>
+      <c r="J17" t="n">
+        <v>60</v>
+      </c>
+      <c r="M17" t="n">
+        <v>10</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Inmediata</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -1167,6 +1274,9 @@
       <c r="L18" t="n">
         <v>10</v>
       </c>
+      <c r="M18" t="n">
+        <v>10</v>
+      </c>
       <c r="P18" t="inlineStr">
         <is>
           <t>Inmediata</t>
@@ -1186,11 +1296,28 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Vista Costanera: Bajan los estacionamientos a 2 x UF 500</t>
-        </is>
+          <t>Vista Costanera</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>12</v>
+      </c>
+      <c r="G19" t="n">
+        <v>10</v>
       </c>
       <c r="H19" t="n">
         <v>100000</v>
+      </c>
+      <c r="J19" t="n">
+        <v>60</v>
+      </c>
+      <c r="M19" t="n">
+        <v>10</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Inmediata</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -1213,7 +1340,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1230,6 +1357,9 @@
         <v>60</v>
       </c>
       <c r="L20" t="n">
+        <v>10</v>
+      </c>
+      <c r="M20" t="n">
         <v>10</v>
       </c>
       <c r="P20" t="inlineStr">
@@ -2720,7 +2850,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H57" t="n">
         <v>0</v>
@@ -2986,7 +3116,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>17.4</v>
+        <v>20</v>
       </c>
       <c r="G64" t="n">
         <v>10</v>
@@ -3067,7 +3197,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="H66" t="n">
         <v>219000</v>
@@ -3103,7 +3233,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="G67" t="n">
         <v>10</v>
@@ -3142,7 +3272,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="G68" t="n">
         <v>10</v>
@@ -3256,7 +3386,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="G71" t="n">
         <v>10</v>
@@ -3415,7 +3545,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H75" t="n">
         <v>203000</v>
@@ -3496,7 +3626,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G77" t="n">
         <v>10</v>
@@ -3586,7 +3716,7 @@
         <v>202000</v>
       </c>
       <c r="J79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M79" t="n">
         <v>8</v>

</xml_diff>

<commit_message>
feat: agrega condiciones comerciales EUROCORP (19 proyectos)
- cc_sync.py: agrega NAME_TO_SLUG para 19 proyectos EUROCORP
- cc_sync.py: agrega parse_euro() y lo incluye en el pipeline
- condiciones_cc_unified.xlsx: 96 proyectos (era 77)
- cc.json / cc_data.js: regenerados con CC EUROCORP

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/viveprop-platform/data/condiciones_cc_unified.xlsx
+++ b/viveprop-platform/data/condiciones_cc_unified.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R79"/>
+  <dimension ref="A1:R98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3732,6 +3732,873 @@
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>proj_santa-elena-1670-mbi</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>EUROCORP</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Santa Elena 1670 MBI</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>2</v>
+      </c>
+      <c r="G80" t="n">
+        <v>10</v>
+      </c>
+      <c r="H80" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J80" t="n">
+        <v>0</v>
+      </c>
+      <c r="N80" t="n">
+        <v>7</v>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>Entrega inmediata</t>
+        </is>
+      </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>4 años de arriendo asegurado y administración gratuita (3%)
+Financiamiento hasta 7% en 48 cuotas sin interés (Pistos) (2%)
+Pago pie hasta 36 cuotas sin intereses (Getnet)
+Dcto máximo sin promociones = 17% (solo para pago de pie contado)
+(Segunda transferencia) (No Fogaes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>proj_vicuna-mackenna-1432</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>EUROCORP</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Vicuña Mackenna 1432</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>4</v>
+      </c>
+      <c r="G81" t="n">
+        <v>10</v>
+      </c>
+      <c r="H81" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J81" t="n">
+        <v>0</v>
+      </c>
+      <c r="N81" t="n">
+        <v>7</v>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>Entrega inmediata</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>4 años de arriendo asegurado y administración gratuita (3%)
+Todos los deptos 1d1b a UF 3.400
+Dcto base 4,0% (no aplica a los 1d1b)
+Financiamiento hasta 7% en 48 cuotas sin interés (Pistos) (2%)
+Pago pie hasta 18 cuotas sin intereses (TC)
+Dcto máximo sin promociones = 19% (solo para pago de pie contado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>proj_mapocho-3521</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>EUROCORP</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Mapocho Torre A y B</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>4</v>
+      </c>
+      <c r="G82" t="n">
+        <v>15</v>
+      </c>
+      <c r="H82" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J82" t="n">
+        <v>0</v>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>Entrega inmediata</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>4 años de arriendo asegurado y administración gratuita (3%)
+Pago pie hasta 36 cuotas sin intereses (Getnet)
+Dcto máximo sin promociones = 22%</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>proj_edificio-mapocho-3521-edificio-a</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>EUROCORP</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Mapocho Torre A y B</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>4</v>
+      </c>
+      <c r="G83" t="n">
+        <v>15</v>
+      </c>
+      <c r="H83" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J83" t="n">
+        <v>0</v>
+      </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>Entrega inmediata</t>
+        </is>
+      </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>4 años de arriendo asegurado y administración gratuita (3%)
+Pago pie hasta 36 cuotas sin intereses (Getnet)
+Dcto máximo sin promociones = 22%</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>proj_rosas-1444</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>EUROCORP</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Rosas 1444</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>7</v>
+      </c>
+      <c r="G84" t="n">
+        <v>10</v>
+      </c>
+      <c r="H84" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J84" t="n">
+        <v>0</v>
+      </c>
+      <c r="N84" t="n">
+        <v>7</v>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>Entrega inmediata</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>4 años de arriendo asegurado y administración gratuita (3%)
+Financiamiento hasta 7% en 48 cuotas sin interés (Pistos) (2%)
+Pago pie hasta 36 cuotas sin intereses (Getnet)
+Dcto máximo sin promociones = 22%</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>proj_guillermo-mann-1401</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>EUROCORP</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Guillermo Mann</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>3</v>
+      </c>
+      <c r="G85" t="n">
+        <v>10</v>
+      </c>
+      <c r="H85" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J85" t="n">
+        <v>0</v>
+      </c>
+      <c r="N85" t="n">
+        <v>7</v>
+      </c>
+      <c r="O85" t="n">
+        <v>7</v>
+      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>Entrega inmediata</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>4 años de arriendo asegurado y administración gratuita (3%)
+PRECIO ESPECIAL 2D1B (4C) UF 4.000
+Financiamiento hasta 7% en 48 cuotas sin interés (Pistos) (2%)
+Pie 7% a 18 cuotas TC
+Dcto máximo sin promociones = 18%</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>proj_independencia-4745</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>EUROCORP</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Independencia 4745</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>4</v>
+      </c>
+      <c r="G86" t="n">
+        <v>15</v>
+      </c>
+      <c r="H86" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J86" t="n">
+        <v>0</v>
+      </c>
+      <c r="O86" t="n">
+        <v>7</v>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>Entrega inmediata</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>4 años de arriendo asegurado y administración gratuita (3%)
+Pie 7% a 18 cuotas TC
+Dcto máximo sin promociones = 22%
+(Actualización de precios febrero 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>proj_jose-pedro-alessandri-1498</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>EUROCORP</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>José Pedro Alessandri</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>7</v>
+      </c>
+      <c r="G87" t="n">
+        <v>3</v>
+      </c>
+      <c r="H87" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J87" t="n">
+        <v>0</v>
+      </c>
+      <c r="M87" t="n">
+        <v>5</v>
+      </c>
+      <c r="N87" t="n">
+        <v>12</v>
+      </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>Entrega inmediata</t>
+        </is>
+      </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>4 años de arriendo asegurado y administración gratuita (3%)
+Upfront del 3,0%, 12% en 48 cuotas con crédito directo, 5% contra escritura
+Pago pie hasta 36 cuotas sin intereses (Getnet)
+Dcto máximo sin promociones = 12%
+*El crédito directo aplica solo si va con arriendo garantizado</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>proj_edificio-vitro</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>EUROCORP</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Vitro</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>5</v>
+      </c>
+      <c r="G88" t="n">
+        <v>3</v>
+      </c>
+      <c r="H88" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J88" t="n">
+        <v>0</v>
+      </c>
+      <c r="M88" t="n">
+        <v>5</v>
+      </c>
+      <c r="N88" t="n">
+        <v>12</v>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>Entrega inmediata</t>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>4 años de arriendo asegurado y administración gratuita (3%)
+Upfront del 3,0%, 12% en 48 cuotas con crédito directo, 5% contra escritura
+Dcto máximo sin promociones = 10%
+*El crédito directo aplica solo si va con arriendo garantizado
+(Segunda transferencia) (No Fogaes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>proj_froilan-roa-5731</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>EUROCORP</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Froilán Roa 5731 – TS y TN</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>8</v>
+      </c>
+      <c r="G89" t="n">
+        <v>5</v>
+      </c>
+      <c r="H89" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J89" t="n">
+        <v>51</v>
+      </c>
+      <c r="M89" t="n">
+        <v>12</v>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>2do semestre 2027</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>3 años de arriendo asegurado (2%)
+Con AG: Sin Upfront, 12% Pie en 51 cuotas toku, 5% aporte pie inmobiliaria, 3% contra escritura
+Sin AG: Sin Upfront, 12% Pie en 51 cuotas (15 antes de entrega + 36 cuotón con TC sin interés), 5% aporte, 3% contra escritura</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>proj_froilan-roa-5731-torre-norte</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>EUROCORP</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Froilán Roa 5731 – TS y TN</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>8</v>
+      </c>
+      <c r="G90" t="n">
+        <v>5</v>
+      </c>
+      <c r="H90" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J90" t="n">
+        <v>51</v>
+      </c>
+      <c r="M90" t="n">
+        <v>12</v>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>2do semestre 2027</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>3 años de arriendo asegurado (2%)
+Con AG: Sin Upfront, 12% Pie en 51 cuotas toku, 5% aporte pie inmobiliaria, 3% contra escritura
+Sin AG: Sin Upfront, 12% Pie en 51 cuotas (15 antes de entrega + 36 cuotón con TC sin interés), 5% aporte, 3% contra escritura</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>proj_diagonal-vicuna</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>EUROCORP</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Diagonal Vicuña Torre Sur</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>5</v>
+      </c>
+      <c r="G91" t="n">
+        <v>5</v>
+      </c>
+      <c r="H91" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J91" t="n">
+        <v>47</v>
+      </c>
+      <c r="M91" t="n">
+        <v>12</v>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>1er semestre 2027</t>
+        </is>
+      </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>3 años de arriendo asegurado (2%)
+Con AG: Sin Upfront, 12% Pie en 47 cuotas toku, 5% aporte pie inmobiliaria, 3% contra escritura
+Sin AG: Sin Upfront, 12% Pie en 47 cuotas (11 antes de entrega + 36 cuotón con TC sin interés), 5% aporte, 3% contra escritura</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>proj_entre-vicunas</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>EUROCORP</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Entre Vicuñas</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>6</v>
+      </c>
+      <c r="G92" t="n">
+        <v>5</v>
+      </c>
+      <c r="H92" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J92" t="n">
+        <v>51</v>
+      </c>
+      <c r="M92" t="n">
+        <v>10</v>
+      </c>
+      <c r="O92" t="n">
+        <v>2</v>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>1er semestre 2027</t>
+        </is>
+      </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>3 años de arriendo asegurado (2%)
+Con AG: Upfront del 2%, 10% del pie en 51 cuotas toku, 5% aporte pie inmobiliaria, 3% contra escritura
+Sin AG: Upfront del 2%, 10% del pie en 51 cuotas (15 antes de entrega + 36 cuotón con TC sin interés), 5% aporte, 3% contra escritura</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>proj_edificio-don-pepe-154</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>EUROCORP</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Don Pepe 2</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>5</v>
+      </c>
+      <c r="G93" t="n">
+        <v>5</v>
+      </c>
+      <c r="H93" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J93" t="n">
+        <v>57</v>
+      </c>
+      <c r="M93" t="n">
+        <v>10</v>
+      </c>
+      <c r="O93" t="n">
+        <v>2</v>
+      </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>1er semestre 2028</t>
+        </is>
+      </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>3 años de arriendo asegurado (2%)
+Con AG: Upfront del 2,0%, 10% Pie en 57 cuotas toku, 5% aporte pie inmobiliaria, 3% contra escritura
+Sin AG: Upfront del 2,0%, 10% Pie en 57 cuotas (21 antes de entrega + 36 cuotón con TC sin interés), 5% aporte, 3% contra escritura</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>proj_edificio-plaza-de-lourdes</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>EUROCORP</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Plaza de Lourdes</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>8</v>
+      </c>
+      <c r="G94" t="n">
+        <v>5</v>
+      </c>
+      <c r="H94" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J94" t="n">
+        <v>57</v>
+      </c>
+      <c r="M94" t="n">
+        <v>12</v>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>1er semestre 2028</t>
+        </is>
+      </c>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>3 años de arriendo asegurado (2%)
+Con AG: Sin Upfront, 12% Pie en 57 cuotas toku, 5% aporte pie inmobiliaria, 3% contra escritura
+Sin AG: Sin Upfront, 12% Pie en 57 cuotas (21 antes de entrega + 36 cuotón con TC sin interés), 5% aporte, 3% contra escritura</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>proj_mirador-irarrazaval</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>EUROCORP</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Mirador Irarrázaval</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>5</v>
+      </c>
+      <c r="G95" t="n">
+        <v>5</v>
+      </c>
+      <c r="H95" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J95" t="n">
+        <v>63</v>
+      </c>
+      <c r="M95" t="n">
+        <v>10</v>
+      </c>
+      <c r="O95" t="n">
+        <v>3</v>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>2do semestre 2028</t>
+        </is>
+      </c>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>3 años de arriendo asegurado (2%)
+Con AG: Upfront del 3,0%, 10% Pie en 63 cuotas toku, 5% aporte pie inmobiliaria, 2% contra escritura
+Sin AG: Upfront del 3,0%, 10% Pie en 63 cuotas (27 antes de entrega + 36 cuotón con TC sin interés), 5% aporte, 2% contra escritura</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>proj_alto-irarrazaval</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>EUROCORP</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Alto Irarrázaval</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>5</v>
+      </c>
+      <c r="G96" t="n">
+        <v>5</v>
+      </c>
+      <c r="H96" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J96" t="n">
+        <v>61</v>
+      </c>
+      <c r="M96" t="n">
+        <v>10</v>
+      </c>
+      <c r="O96" t="n">
+        <v>3</v>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>2do semestre 2028</t>
+        </is>
+      </c>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>3 años de arriendo asegurado (2%)
+Con AG: Upfront del 3,0%, 10% Pie en 61 cuotas toku, 5% aporte pie inmobiliaria, 2% contra escritura
+Sin AG: Upfront del 3,0%, 10% Pie en 61 cuotas (25 antes de entrega + 36 cuotón con TC sin interés), 5% aporte, 2% contra escritura</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>proj_edificio-ambar-urbano</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>EUROCORP</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Ambar</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>5</v>
+      </c>
+      <c r="G97" t="n">
+        <v>5</v>
+      </c>
+      <c r="H97" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J97" t="n">
+        <v>61</v>
+      </c>
+      <c r="M97" t="n">
+        <v>12</v>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>2do semestre 2028</t>
+        </is>
+      </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>3 años de arriendo asegurado (2%)
+Con AG: Sin Upfront, 12% Pie en 61 cuotas toku, 5% aporte pie inmobiliaria, 3% contra escritura
+Sin AG: Sin Upfront, 12% Pie en 61 cuotas (25 antes de entrega + 36 cuotón con TC sin interés), 5% aporte, 3% contra escritura</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>proj_nova-parque</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>EUROCORP</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Nova Parque</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>5</v>
+      </c>
+      <c r="G98" t="n">
+        <v>5</v>
+      </c>
+      <c r="H98" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J98" t="n">
+        <v>58</v>
+      </c>
+      <c r="M98" t="n">
+        <v>10</v>
+      </c>
+      <c r="O98" t="n">
+        <v>3</v>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>1er semestre 2028</t>
+        </is>
+      </c>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>3 años de arriendo asegurado (2%)
+Con AG: Upfront del 3,0%, 10% Pie en 58 cuotas toku, 5% aporte pie inmobiliaria, 2% contra escritura
+Sin AG: Upfront del 3,0%, 10% Pie en 58 cuotas (22 antes de entrega + 36 cuotón con TC sin interés), 5% aporte, 2% contra escritura</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>